<commit_message>
pretty good id say soo
</commit_message>
<xml_diff>
--- a/flex.xlsx
+++ b/flex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Mega\Projects\Python\whyflexgood\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8E164D-A311-4109-AF88-8FC76CF18EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B87DC0-24B4-453B-8B38-59A2EEAB1F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="3420" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -528,11 +528,10 @@
     <t>prevent</t>
   </si>
   <si>
-    <t xml:space="preserve">how
-</t>
-  </si>
-  <si>
     <t>feel</t>
+  </si>
+  <si>
+    <t>how</t>
   </si>
 </sst>
 </file>
@@ -690,7 +689,7 @@
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="when" dataDxfId="4"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="what" dataDxfId="3"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="prevent" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="how_x000a_" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="how" dataDxfId="1"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="feel" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -995,12 +994,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G129"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="7" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>161</v>
       </c>
@@ -1017,13 +1016,13 @@
         <v>165</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="G1" t="s">
         <v>166</v>
       </c>
-      <c r="G1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1043,7 +1042,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1063,7 +1062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1086,7 +1085,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1126,7 +1125,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1148,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1172,7 +1171,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1195,7 +1194,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -1215,7 +1214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1235,7 +1234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1255,7 +1254,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1275,7 +1274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1298,7 +1297,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1321,7 +1320,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1367,7 +1366,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -1390,7 +1389,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -1410,7 +1409,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -1430,7 +1429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -1450,7 +1449,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1473,7 +1472,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>5</v>
       </c>
@@ -1493,7 +1492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -1516,7 +1515,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1536,7 +1535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -1559,7 +1558,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -1579,7 +1578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>5</v>
       </c>
@@ -1599,7 +1598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -1622,7 +1621,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>5</v>
       </c>
@@ -1645,7 +1644,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -1668,7 +1667,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -1688,7 +1687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
@@ -1708,7 +1707,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -1728,7 +1727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -1748,7 +1747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -1768,7 +1767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>0</v>
       </c>
@@ -1788,7 +1787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -1811,7 +1810,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>29</v>
       </c>
@@ -1834,7 +1833,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -1854,7 +1853,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -1874,7 +1873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>0</v>
       </c>
@@ -1894,7 +1893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -1914,7 +1913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>81</v>
       </c>
@@ -1934,7 +1933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>81</v>
       </c>
@@ -1954,7 +1953,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>81</v>
       </c>
@@ -1974,7 +1973,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>81</v>
       </c>
@@ -1997,7 +1996,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -2017,7 +2016,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>5</v>
       </c>
@@ -2040,7 +2039,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>40</v>
       </c>
@@ -2060,7 +2059,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>0</v>
       </c>
@@ -2083,7 +2082,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>40</v>
       </c>
@@ -2103,7 +2102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>5</v>
       </c>
@@ -2126,7 +2125,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>40</v>
       </c>
@@ -2146,7 +2145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>5</v>
       </c>
@@ -2166,7 +2165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>40</v>
       </c>
@@ -2189,7 +2188,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>5</v>
       </c>
@@ -2212,7 +2211,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>5</v>
       </c>
@@ -2232,7 +2231,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>5</v>
       </c>
@@ -2252,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>29</v>
       </c>
@@ -2272,7 +2271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>29</v>
       </c>
@@ -2292,7 +2291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>40</v>
       </c>
@@ -2312,7 +2311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>5</v>
       </c>
@@ -2335,7 +2334,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -2358,7 +2357,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>5</v>
       </c>
@@ -2378,7 +2377,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>5</v>
       </c>
@@ -2398,7 +2397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>5</v>
       </c>
@@ -2421,7 +2420,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>29</v>
       </c>
@@ -2444,7 +2443,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>29</v>
       </c>
@@ -2464,7 +2463,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>81</v>
       </c>
@@ -2487,7 +2486,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>81</v>
       </c>
@@ -2510,7 +2509,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>0</v>
       </c>
@@ -2530,7 +2529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>29</v>
       </c>
@@ -2553,7 +2552,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>29</v>
       </c>
@@ -2573,7 +2572,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>5</v>
       </c>
@@ -2593,7 +2592,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>81</v>
       </c>
@@ -2616,7 +2615,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>40</v>
       </c>
@@ -2639,7 +2638,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>40</v>
       </c>
@@ -2662,7 +2661,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>5</v>
       </c>
@@ -2682,7 +2681,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>40</v>
       </c>
@@ -2702,7 +2701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>40</v>
       </c>
@@ -2722,7 +2721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>29</v>
       </c>
@@ -2742,7 +2741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>81</v>
       </c>
@@ -2762,7 +2761,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>29</v>
       </c>
@@ -2782,7 +2781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>29</v>
       </c>
@@ -2802,7 +2801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>81</v>
       </c>
@@ -2825,7 +2824,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>5</v>
       </c>
@@ -2848,7 +2847,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>81</v>
       </c>
@@ -2871,7 +2870,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>81</v>
       </c>
@@ -2894,7 +2893,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>81</v>
       </c>
@@ -2914,7 +2913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>81</v>
       </c>
@@ -2934,7 +2933,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>29</v>
       </c>
@@ -2957,7 +2956,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>81</v>
       </c>
@@ -2980,7 +2979,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>0</v>
       </c>
@@ -3000,7 +2999,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>81</v>
       </c>
@@ -3023,7 +3022,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>81</v>
       </c>
@@ -3046,7 +3045,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>81</v>
       </c>
@@ -3069,7 +3068,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>0</v>
       </c>
@@ -3092,7 +3091,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>5</v>
       </c>
@@ -3112,7 +3111,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>5</v>
       </c>
@@ -3132,7 +3131,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>0</v>
       </c>
@@ -3155,7 +3154,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>81</v>
       </c>
@@ -3178,7 +3177,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>81</v>
       </c>
@@ -3201,7 +3200,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>29</v>
       </c>
@@ -3224,7 +3223,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>0</v>
       </c>
@@ -3244,7 +3243,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>0</v>
       </c>
@@ -3264,7 +3263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>0</v>
       </c>
@@ -3284,7 +3283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>0</v>
       </c>
@@ -3307,7 +3306,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>81</v>
       </c>
@@ -3330,7 +3329,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>81</v>
       </c>
@@ -3353,7 +3352,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>81</v>
       </c>
@@ -3376,7 +3375,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>81</v>
       </c>
@@ -3399,7 +3398,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>81</v>
       </c>
@@ -3419,7 +3418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>81</v>
       </c>
@@ -3439,7 +3438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>81</v>
       </c>
@@ -3459,7 +3458,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>29</v>
       </c>
@@ -3482,7 +3481,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>29</v>
       </c>
@@ -3502,7 +3501,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>29</v>
       </c>
@@ -3525,7 +3524,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>0</v>
       </c>
@@ -3545,7 +3544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>5</v>
       </c>
@@ -3565,7 +3564,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>0</v>
       </c>
@@ -3588,7 +3587,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>40</v>
       </c>
@@ -3611,7 +3610,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>29</v>
       </c>
@@ -3634,7 +3633,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>29</v>
       </c>
@@ -3654,7 +3653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>29</v>
       </c>
@@ -3677,7 +3676,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>40</v>
       </c>
@@ -3700,7 +3699,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>29</v>
       </c>
@@ -3720,7 +3719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>29</v>
       </c>
@@ -3743,7 +3742,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>81</v>
       </c>

</xml_diff>